<commit_message>
research: classify Diwali Muhurat sessions in calendar audit
</commit_message>
<xml_diff>
--- a/research/output/complement_strategy/eligibility_audit.xlsx
+++ b/research/output/complement_strategy/eligibility_audit.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Eligibility_audit" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Muhurat_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Original_audit" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,6 +415,1242 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:S12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Eligibility_reason</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Opening_rows</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Valid_opening_seconds_if_measured</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Observed_expiries</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tick_size</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Tick_mtime_ns</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Original_exception</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>File_first_source_time</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>File_last_source_time</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Raw_eligibility_reason</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Session_type</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Eligibility_class</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Scheduled_open</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Scheduled_close</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Circular</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Source_URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2021-11-04</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Diwali/Muhurat scheduled session outside fixed morning strategy window</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11101782</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>1769700420868047300</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ValueError: No expiry observed before09:30 at least2calendar days ahead</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1900-01-01 18:15:00</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>1900-01-01 19:15:01</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>No morning observations</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Scheduled_session_outside_policy_window</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>18:15:00</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>19:15:00</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/50049</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2021-10-21</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>https://archives.nseindia.com/content/circulars/FAOP50049.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2022-10-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Diwali/Muhurat scheduled session outside fixed morning strategy window</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14122873</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1766608535070833900</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ValueError: No expiry observed before09:30 at least2calendar days ahead</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1900-01-01 18:15:00</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1900-01-01 19:15:02</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>No morning observations</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Scheduled_session_outside_policy_window</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>18:15:00</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>19:15:00</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/54024</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2022-10-11</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>https://archives.nseindia.com/content/circulars/FAOP54024.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2023-11-12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Diwali/Muhurat scheduled session outside fixed morning strategy window</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10843966</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1766604186561964700</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ValueError: No expiry observed before09:30 at least2calendar days ahead</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1900-01-01 18:15:00</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1900-01-01 19:15:02</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>No morning observations</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Scheduled_session_outside_policy_window</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>18:15:00</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>19:15:00</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/59126</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2023-10-27</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/circulars/FAOP59126.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-07-05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>185492</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>108819450</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1769703541411408500</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TypeError: ufunc 'isfinite' not supported for the input types, and the inputs could not be safely coerced to any supported types according to the casting rule ''safe''</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1900-01-01 09:15:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1900-01-01 15:33:47</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Not_classified_by_this_reference</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Missing_underlying_data</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-08-20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>150489</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" t="n">
+        <v>106551999</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1769102455806700900</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TypeError: ufunc 'isfinite' not supported for the input types, and the inputs could not be safely coerced to any supported types according to the casting rule ''safe''</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1900-01-01 09:15:00</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1900-01-01 15:30:35</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Not_classified_by_this_reference</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Missing_underlying_data</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2024-11-01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Diwali/Muhurat scheduled session outside fixed morning strategy window</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>12537642</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1769688267697433800</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ValueError: No expiry observed before09:30 at least2calendar days ahead</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1900-01-01 18:00:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1900-01-01 19:00:10</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>No morning observations</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Scheduled_session_outside_policy_window</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>18:00:00</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>19:00:00</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/64630</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2024-10-19</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/circulars/FAOP64630.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-10-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Diwali/Muhurat scheduled session outside fixed morning strategy window</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>38898809</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1766599409220879100</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ValueError: No expiry observed before09:30 at least2calendar days ahead</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1900-01-01 13:45:00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1900-01-01 14:45:02</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>No morning observations</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Scheduled_session_outside_policy_window</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/70320</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2025-09-22</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/circulars/FAOP70320.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>235201</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>11</v>
+      </c>
+      <c r="F9" t="n">
+        <v>166679482</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1766620862948690200</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TypeError: ufunc 'isfinite' not supported for the input types, and the inputs could not be safely coerced to any supported types according to the casting rule ''safe''</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1900-01-01 09:15:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1900-01-01 15:31:12</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Not_classified_by_this_reference</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Missing_underlying_data</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>315696</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" t="n">
+        <v>240267600</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1777462688438203900</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TypeError: ufunc 'isfinite' not supported for the input types, and the inputs could not be safely coerced to any supported types according to the casting rule ''safe''</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1900-01-01 09:15:00</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1900-01-01 15:31:44</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Not_classified_by_this_reference</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Missing_underlying_data</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1494</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1115490</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1781197398165800100</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>TypeError: ufunc 'isfinite' not supported for the input types, and the inputs could not be safely coerced to any supported types according to the casting rule ''safe''</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1900-01-01 09:00:00</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1900-01-01 15:30:01</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>UnderlyingLTP is Arrow null type for entire source file</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Not_classified_by_this_reference</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Missing_underlying_data</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fewer than600 valid opening underlying seconds</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>157389</v>
+      </c>
+      <c r="D12" t="n">
+        <v>477</v>
+      </c>
+      <c r="E12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" t="n">
+        <v>385203018</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1790850156761470100</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>ValueError: Insufficient opening underlying coverage</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1900-01-01 09:00:01</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1900-01-01 15:40:02</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Fewer than600 valid opening underlying seconds</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Not_classified_by_this_reference</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Insufficient_opening_data</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Session_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Timezone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Scheduled_open</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Scheduled_close</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Circular</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Source_URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2021-11-04</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>18:15:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>19:15:00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/50049</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2021-10-21</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://archives.nseindia.com/content/circulars/FAOP50049.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2022-10-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>18:15:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>19:15:00</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/54024</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2022-10-11</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://archives.nseindia.com/content/circulars/FAOP54024.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2023-11-12</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>18:15:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>19:15:00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/59126</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2023-10-27</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/circulars/FAOP59126.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-11-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>18:00:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>19:00:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/64630</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2024-10-19</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/circulars/FAOP64630.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-10-21</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Diwali_Muhurat</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>14:45:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>NSE/FAOP/70320</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-09-22</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://nsearchives.nseindia.com/content/circulars/FAOP70320.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>